<commit_message>
City index 26-7 4/11.
</commit_message>
<xml_diff>
--- a/data_indexpoints_tidy/tallmateriale_16952.xlsx
+++ b/data_indexpoints_tidy/tallmateriale_16952.xlsx
@@ -3344,12 +3344,6 @@
       <c r="E5">
         <v>2026</v>
       </c>
-      <c r="F5">
-        <v>7.28</v>
-      </c>
-      <c r="G5">
-        <v>8.15</v>
-      </c>
     </row>
     <row r="6" spans="1:17">
       <c r="A6" t="s">
@@ -5305,12 +5299,6 @@
       <c r="E57">
         <v>2026</v>
       </c>
-      <c r="H57">
-        <v>2.63</v>
-      </c>
-      <c r="I57">
-        <v>8.039999999999999</v>
-      </c>
       <c r="J57">
         <v>1.93</v>
       </c>
@@ -6861,12 +6849,6 @@
       <c r="E97">
         <v>2026</v>
       </c>
-      <c r="F97">
-        <v>1.57</v>
-      </c>
-      <c r="G97">
-        <v>-1.34</v>
-      </c>
     </row>
     <row r="98" spans="1:17">
       <c r="A98" t="s">
@@ -7010,12 +6992,6 @@
       <c r="E101">
         <v>2026</v>
       </c>
-      <c r="F101">
-        <v>6.53</v>
-      </c>
-      <c r="G101">
-        <v>10.26</v>
-      </c>
     </row>
     <row r="102" spans="1:17">
       <c r="A102" t="s">
@@ -7158,12 +7134,6 @@
       </c>
       <c r="E105">
         <v>2026</v>
-      </c>
-      <c r="F105">
-        <v>7.22</v>
-      </c>
-      <c r="G105">
-        <v>8.869999999999999</v>
       </c>
     </row>
     <row r="106" spans="1:17">
@@ -7355,9 +7325,6 @@
       <c r="F2">
         <v>3.29</v>
       </c>
-      <c r="H2">
-        <v>7.7</v>
-      </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
@@ -7634,7 +7601,7 @@
         <v>7.77</v>
       </c>
       <c r="H15">
-        <v>4.07</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -7845,9 +7812,6 @@
       <c r="G25">
         <v>-5.16</v>
       </c>
-      <c r="H25">
-        <v>0.15</v>
-      </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
@@ -7871,9 +7835,6 @@
       <c r="G26">
         <v>9.08</v>
       </c>
-      <c r="H26">
-        <v>8.32</v>
-      </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
@@ -7896,9 +7857,6 @@
       </c>
       <c r="G27">
         <v>9.300000000000001</v>
-      </c>
-      <c r="H27">
-        <v>8.01</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -8153,22 +8111,22 @@
         <v>188</v>
       </c>
       <c r="G6">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="H6">
-        <v>1.0173</v>
+        <v>1.0087</v>
       </c>
       <c r="I6">
-        <v>1.73</v>
+        <v>0.87</v>
       </c>
       <c r="J6">
-        <v>1.107930588530208</v>
+        <v>1.048077636583285</v>
       </c>
       <c r="K6">
-        <v>-0.44</v>
+        <v>-1.18</v>
       </c>
       <c r="L6">
-        <v>3.9</v>
+        <v>2.92</v>
       </c>
       <c r="M6" t="s">
         <v>20</v>

</xml_diff>